<commit_message>
Feat: 0006 : updated tools and packages tracker
</commit_message>
<xml_diff>
--- a/app/LQ/documents/Micro-Services-Packages.xlsx
+++ b/app/LQ/documents/Micro-Services-Packages.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepo\python-documents\documents\architect_solutions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepo\python-stack\app\LQ\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="129">
   <si>
     <t>Category</t>
   </si>
@@ -408,6 +408,11 @@
   </si>
   <si>
     <t>Tools and Packages for Micro Services</t>
+  </si>
+  <si>
+    <t>Open LLMs: Qwen, Mistral, DeepSeek, Gemma.
+Embedding Models: BGE, E5, Nomic Embed, MiniLM.
+LLM runtime : Ollama , VLLM</t>
   </si>
 </sst>
 </file>
@@ -446,7 +451,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -469,35 +474,29 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -779,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.21875" style="1" bestFit="1" customWidth="1"/>
@@ -789,18 +788,23 @@
     <col min="5" max="5" width="35.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="27.109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>127</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -822,8 +826,9 @@
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
@@ -845,8 +850,9 @@
       <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -868,8 +874,9 @@
       <c r="G4" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
@@ -891,8 +898,9 @@
       <c r="G5" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>28</v>
       </c>
@@ -914,8 +922,9 @@
       <c r="G6" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>31</v>
       </c>
@@ -937,8 +946,9 @@
       <c r="G7" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>33</v>
       </c>
@@ -960,8 +970,9 @@
       <c r="G8" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>35</v>
       </c>
@@ -983,8 +994,9 @@
       <c r="G9" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>42</v>
       </c>
@@ -1006,8 +1018,9 @@
       <c r="G10" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
@@ -1029,8 +1042,9 @@
       <c r="G11" s="4" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>54</v>
       </c>
@@ -1052,8 +1066,9 @@
       <c r="G12" s="4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>59</v>
       </c>
@@ -1075,8 +1090,9 @@
       <c r="G13" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>65</v>
       </c>
@@ -1098,8 +1114,9 @@
       <c r="G14" s="4" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>71</v>
       </c>
@@ -1121,8 +1138,9 @@
       <c r="G15" s="4" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>77</v>
       </c>
@@ -1144,8 +1162,9 @@
       <c r="G16" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>82</v>
       </c>
@@ -1167,8 +1186,11 @@
       <c r="G17" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H17" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>88</v>
       </c>
@@ -1190,8 +1212,9 @@
       <c r="G18" s="4" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>92</v>
       </c>
@@ -1213,8 +1236,9 @@
       <c r="G19" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>94</v>
       </c>
@@ -1236,8 +1260,9 @@
       <c r="G20" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>99</v>
       </c>
@@ -1257,8 +1282,9 @@
         <v>102</v>
       </c>
       <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>92</v>
       </c>
@@ -1278,8 +1304,9 @@
         <v>12</v>
       </c>
       <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>94</v>
       </c>
@@ -1299,8 +1326,9 @@
         <v>104</v>
       </c>
       <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>105</v>
       </c>
@@ -1320,8 +1348,9 @@
         <v>110</v>
       </c>
       <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>111</v>
       </c>
@@ -1341,8 +1370,9 @@
         <v>12</v>
       </c>
       <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>113</v>
       </c>
@@ -1362,8 +1392,9 @@
         <v>118</v>
       </c>
       <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H26" s="6"/>
+    </row>
+    <row r="27" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>119</v>
       </c>
@@ -1383,8 +1414,9 @@
         <v>124</v>
       </c>
       <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>125</v>
       </c>
@@ -1404,6 +1436,7 @@
         <v>12</v>
       </c>
       <c r="G28" s="4"/>
+      <c r="H28" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>